<commit_message>
release: V1.8.81 - CRM Header Refactor, Mind Map Enhancements, and PTE Write Essay Topic Filters
</commit_message>
<xml_diff>
--- a/public/database/Write Essay/PTE_453_Cleaned_Prompts_Topics_Task_Types.xlsx
+++ b/public/database/Write Essay/PTE_453_Cleaned_Prompts_Topics_Task_Types.xlsx
@@ -556,14 +556,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>453 Cleaned PTE Write Essay Prompts</t>
+          <t>453 Cleaned PTE Write Essay Prompts (3-Model Verified)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each prompt is shown with its single task type, one primary topic, and up to two secondary topics.</t>
+          <t>Each prompt is verified by 3 Local LLMs (Gemma 4, Qwen 3, DeepSeek-R1) with single task type and up to 3 topic tags.</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>"The only thing that interferes with my learning is education." - Albert Einstein. What did he mean by that? Do you think he is correct?</t>
+          <t>“The only thing that interferes with my learning is education.” – Albert Einstein. What did he mean by that? Do you think he is correct?</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Advertisements make people purchase things they don't need or cannot afford, but they also convey information to increase people's life quality. What is your opinion?</t>
+          <t>Advertisements make people purchase things they don’t need or cannot afford, but they also convey information to increase people's life quality. What is your opinion?</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Economy, money, and trade</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr"/>
@@ -703,7 +703,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Traffic</t>
+          <t>City development</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -736,8 +736,16 @@
           <t>Government, politics, and diplomacy</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Food and health</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Economy, money, and trade</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -832,7 +840,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -854,7 +862,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -933,7 +941,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr"/>
@@ -955,7 +963,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr"/>
@@ -1011,7 +1019,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>'In a war of ideas, it is people who get killed'. Does a common man suffer from a group's ideology? Express your opinion and support the same with reasons and examples.</t>
+          <t>'In a war of ideas, it is people who get killed'. Does a common man suffer from a group’s ideology? Express your opinion and support the same with reasons and examples.</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1024,8 +1032,16 @@
           <t>Socio-cultural and global issues</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="7" t="inlineStr"/>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Ethics</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Government, politics, and diplomacy</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -1069,7 +1085,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Government, politics, and diplomacy</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr"/>
@@ -1091,7 +1107,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Socio-cultural and global issues</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr"/>
@@ -1174,7 +1190,7 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -1205,7 +1221,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr"/>
@@ -1227,11 +1243,19 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr"/>
-      <c r="F31" s="7" t="inlineStr"/>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -1249,7 +1273,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Art and museums</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr"/>
@@ -1266,7 +1290,7 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -1323,12 +1347,12 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
           <t>Language</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>Education</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -1348,7 +1372,7 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -1379,7 +1403,7 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Travelling and tourism</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr"/>
@@ -1391,7 +1415,7 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Many workers like nurses and teachers should get more pay, especially in recent years when people in finance，film actors and company leaders are paid a larger amount of money. To what extent do you agree or disagree with the above statement and what's your opinion?</t>
+          <t>Many workers like nurses and teachers should get more pay, especially in recent years when people in finance，film actors and company leaders are paid a larger amount of money. To what extent do you agree or disagree with the above statement and what’s your opinion?</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -1401,7 +1425,7 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -1487,7 +1511,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Media and communication</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr"/>
@@ -1521,12 +1545,12 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Nowadays, it is increasingly more difficult to maintain the right balance between work and the other aspects of one's life, such as leisure pursuits with family members. How important do you think this balance is? What are the reasons that make some people think that this is hard to achieve？</t>
+          <t>Nowadays, it is increasingly more difficult to maintain the right balance between work and the other aspects of one’s life, such as leisure pursuits with family members. How important do you think this balance is? What are the reasons that make some people think that this is hard to achieve？</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -1557,7 +1581,7 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr"/>
@@ -1601,12 +1625,12 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
+          <t>City development</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
           <t>Population</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>City development</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr"/>
@@ -1627,12 +1651,12 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
+          <t>Crime, punishment, and law</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
           <t>Age, generation, and gender</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>Crime, punishment, and law</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
@@ -1652,12 +1676,12 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -1687,12 +1711,12 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
+          <t>Art and museums</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="inlineStr">
-        <is>
-          <t>Art and museums</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr"/>
@@ -1735,7 +1759,7 @@
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Traffic</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -1827,11 +1851,19 @@
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
           <t>Art and museums</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr"/>
-      <c r="F55" s="7" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n">
@@ -1849,7 +1881,7 @@
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr"/>
@@ -1871,7 +1903,7 @@
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Media and communication</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr"/>
@@ -1927,17 +1959,17 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Some people said creativity is something a person was born with. Others thought creativity can be taught and developed. What's your opinion? Explain.</t>
+          <t>Some people said creativity is something a person was born with. Others thought creativity can be taught and developed. What’s your opinion? Explain.</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>To what extent do you agree or disagree</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Art and museums</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr"/>
@@ -1981,15 +2013,19 @@
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
+          <t>Ethics</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E62" s="7" t="inlineStr">
-        <is>
-          <t>Economy, money, and trade</t>
-        </is>
-      </c>
-      <c r="F62" s="7" t="inlineStr"/>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>Media and communication</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
@@ -2085,7 +2121,7 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>Space travel is fantastic these days, but there are many issues - such as environmental problems - that we should be focusing on. What are your views on the allocation of public funding to space travel?</t>
+          <t>Space travel is fantastic these days, but there are many issues – such as environmental problems – that we should be focusing on. What are your views on the allocation of public funding to space travel?</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
@@ -2095,7 +2131,7 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Government, politics, and diplomacy</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr"/>
@@ -2107,7 +2143,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Sports and games create disturbance in students' life because students cannot fully concentrate on their studies. To what extent do you agree or disagree?</t>
+          <t>Sports and games create disturbance in students’ life because students cannot fully concentrate on their studies. To what extent do you agree or disagree?</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
@@ -2159,7 +2195,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Some say that in today's world the value of humanities has been eclipsed by the necessity of preparing for specific wealth-producing careers, such as medicine. What is your opinion about a role in today's changing world for study of the humanities?</t>
+          <t>Some say that in today’s world the value of humanities has been eclipsed by the necessity of preparing for specific wealth-producing careers, such as medicine. What is your opinion about a role in today’s changing world for study of the humanities?</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
@@ -2169,7 +2205,7 @@
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Socio-cultural and global issues</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr"/>
@@ -2191,7 +2227,7 @@
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Leisure, sports, and hobbies</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr"/>
@@ -2208,7 +2244,7 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -2235,7 +2271,7 @@
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Economy, money, and trade</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr"/>
@@ -2257,7 +2293,7 @@
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr"/>
@@ -2274,7 +2310,7 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
@@ -2296,7 +2332,7 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -2357,7 +2393,7 @@
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr"/>
@@ -2374,7 +2410,7 @@
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
@@ -2448,7 +2484,7 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
@@ -2497,7 +2533,7 @@
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr"/>
@@ -2536,7 +2572,7 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
@@ -2563,11 +2599,19 @@
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
           <t>Ethics</t>
         </is>
       </c>
-      <c r="E87" s="7" t="inlineStr"/>
-      <c r="F87" s="7" t="inlineStr"/>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n">
@@ -2607,7 +2651,7 @@
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Media and communication</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr"/>
@@ -2624,7 +2668,7 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
@@ -2673,7 +2717,7 @@
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr"/>
@@ -2717,12 +2761,12 @@
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
+          <t>City development</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
           <t>Population</t>
-        </is>
-      </c>
-      <c r="E94" s="7" t="inlineStr">
-        <is>
-          <t>City development</t>
         </is>
       </c>
       <c r="F94" s="7" t="inlineStr"/>
@@ -2743,7 +2787,7 @@
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr"/>
@@ -2777,7 +2821,7 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>"National happiness index" has better performance than economic increase in a nation's development. Do you agree and how to measure "national happiness"?</t>
+          <t>"National happiness index" has better performance than economic increase in a nation’s development. Do you agree and how to measure "national happiness"?</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -2787,7 +2831,7 @@
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr"/>
@@ -2804,12 +2848,12 @@
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr"/>
@@ -2826,16 +2870,24 @@
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
           <t>Lifestyle</t>
         </is>
       </c>
-      <c r="E99" s="7" t="inlineStr"/>
-      <c r="F99" s="7" t="inlineStr"/>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>Science, technology, and innovation</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="n">
@@ -2870,12 +2922,12 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>Socio-cultural and global issues</t>
+          <t>Government, politics, and diplomacy</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr"/>
@@ -2922,12 +2974,12 @@
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Food and health</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr"/>
@@ -2952,8 +3004,16 @@
           <t>Traffic</t>
         </is>
       </c>
-      <c r="E104" s="7" t="inlineStr"/>
-      <c r="F104" s="7" t="inlineStr"/>
+      <c r="E104" s="7" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="F104" s="7" t="inlineStr">
+        <is>
+          <t>City development</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="n">
@@ -2992,7 +3052,7 @@
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -3014,7 +3074,7 @@
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
@@ -3041,7 +3101,7 @@
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>Economy, money, and trade</t>
+          <t>Government, politics, and diplomacy</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr"/>
@@ -3063,7 +3123,7 @@
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr"/>
@@ -3080,7 +3140,7 @@
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -3181,7 +3241,7 @@
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr"/>
@@ -3220,12 +3280,12 @@
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>Discuss both views and give your opinions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr"/>
@@ -3247,12 +3307,12 @@
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
           <t>Food and health</t>
-        </is>
-      </c>
-      <c r="E117" s="7" t="inlineStr">
-        <is>
-          <t>Lifestyle</t>
         </is>
       </c>
       <c r="F117" s="7" t="inlineStr"/>
@@ -3273,7 +3333,7 @@
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Government, politics, and diplomacy</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
@@ -3299,7 +3359,7 @@
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>Traffic</t>
+          <t>City development</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr"/>
@@ -3316,7 +3376,7 @@
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
@@ -3447,7 +3507,7 @@
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr"/>
@@ -3469,7 +3529,7 @@
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>Art and museums</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr"/>
@@ -3491,7 +3551,7 @@
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>Travelling and tourism</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr"/>
@@ -3503,7 +3563,7 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>There are more men or women in certain jobs and there's nothing we can change about it. Do you agree with that?</t>
+          <t>There are more men or women in certain jobs and there’s nothing we can change about it. Do you agree with that?</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
@@ -3513,7 +3573,7 @@
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Age, generation, and gender</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr"/>
@@ -3535,7 +3595,7 @@
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>Government, politics, and diplomacy</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr"/>
@@ -3579,7 +3639,7 @@
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr"/>
@@ -3591,7 +3651,7 @@
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>Which one has the greater impact on human's life, aeroplanes or cars?</t>
+          <t>Which one has the greater impact on human’s life, aeroplanes or cars?</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
@@ -3675,7 +3735,7 @@
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>Art and museums</t>
+          <t>Government, politics, and diplomacy</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr"/>
@@ -3697,12 +3757,12 @@
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
+          <t>Work</t>
+        </is>
+      </c>
+      <c r="E136" s="7" t="inlineStr">
+        <is>
           <t>Age, generation, and gender</t>
-        </is>
-      </c>
-      <c r="E136" s="7" t="inlineStr">
-        <is>
-          <t>Work</t>
         </is>
       </c>
       <c r="F136" s="7" t="inlineStr"/>
@@ -3745,7 +3805,7 @@
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
@@ -3853,7 +3913,7 @@
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr"/>
@@ -3875,7 +3935,7 @@
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>Art and museums</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr"/>
@@ -4001,7 +4061,7 @@
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr"/>
@@ -4028,12 +4088,12 @@
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
+          <t>Economy, money, and trade</t>
+        </is>
+      </c>
+      <c r="F149" s="7" t="inlineStr">
+        <is>
           <t>Socio-cultural and global issues</t>
-        </is>
-      </c>
-      <c r="F149" s="7" t="inlineStr">
-        <is>
-          <t>Economy, money, and trade</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4113,7 @@
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>Media and communication</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
@@ -4127,12 +4187,12 @@
       </c>
       <c r="D153" s="7" t="inlineStr">
         <is>
+          <t>City development</t>
+        </is>
+      </c>
+      <c r="E153" s="7" t="inlineStr">
+        <is>
           <t>Population</t>
-        </is>
-      </c>
-      <c r="E153" s="7" t="inlineStr">
-        <is>
-          <t>City development</t>
         </is>
       </c>
       <c r="F153" s="7" t="inlineStr"/>
@@ -4153,11 +4213,19 @@
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E154" s="7" t="inlineStr">
+        <is>
+          <t>Age, generation, and gender</t>
+        </is>
+      </c>
+      <c r="F154" s="7" t="inlineStr">
+        <is>
           <t>Media and communication</t>
         </is>
       </c>
-      <c r="E154" s="7" t="inlineStr"/>
-      <c r="F154" s="7" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="5" t="n">
@@ -4187,7 +4255,7 @@
       </c>
       <c r="B156" s="6" t="inlineStr">
         <is>
-          <t>University experience is more important than a university's degree. Some people argue that university life is much more important than an educational degree in job market. Do you agree or disagree?</t>
+          <t>University experience is more important than a university’s degree. Some people argue that university life is much more important than an educational degree in job market. Do you agree or disagree?</t>
         </is>
       </c>
       <c r="C156" s="7" t="inlineStr">
@@ -4222,7 +4290,7 @@
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D157" s="7" t="inlineStr">
@@ -4274,7 +4342,7 @@
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
@@ -4291,7 +4359,7 @@
       </c>
       <c r="B160" s="6" t="inlineStr">
         <is>
-          <t>Nowadays, people believe that the environment influences their accomplishments. Some people think their success and accomplishment were influenced by the places where they grew up. Do you think the environment does or does not affect people's accomplishment and how it affects? Please give an example of a famous person to support your statement.</t>
+          <t>Nowadays, people believe that the environment influences their accomplishments. Some people think their success and accomplishment were influenced by the places where they grew up. Do you think the environment does or does not affect people’s accomplishment and how it affects? Please give an example of a famous person to support your statement.</t>
         </is>
       </c>
       <c r="C160" s="7" t="inlineStr">
@@ -4340,7 +4408,7 @@
       </c>
       <c r="C162" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
@@ -4520,15 +4588,19 @@
       </c>
       <c r="C170" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D170" s="7" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
-        </is>
-      </c>
-      <c r="E170" s="7" t="inlineStr"/>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E170" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
       <c r="F170" s="7" t="inlineStr"/>
     </row>
     <row r="171">
@@ -4564,7 +4636,7 @@
       </c>
       <c r="C172" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D172" s="7" t="inlineStr">
@@ -4595,12 +4667,12 @@
       </c>
       <c r="D173" s="7" t="inlineStr">
         <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E173" s="7" t="inlineStr">
+        <is>
           <t>Language</t>
-        </is>
-      </c>
-      <c r="E173" s="7" t="inlineStr">
-        <is>
-          <t>Education</t>
         </is>
       </c>
       <c r="F173" s="7" t="inlineStr">
@@ -4790,7 +4862,7 @@
       </c>
       <c r="C181" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D181" s="7" t="inlineStr">
@@ -4905,7 +4977,7 @@
       </c>
       <c r="D186" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E186" s="7" t="inlineStr"/>
@@ -4927,7 +4999,7 @@
       </c>
       <c r="D187" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
@@ -5001,12 +5073,12 @@
       </c>
       <c r="D190" s="7" t="inlineStr">
         <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
           <t>Food and health</t>
-        </is>
-      </c>
-      <c r="E190" s="7" t="inlineStr">
-        <is>
-          <t>Lifestyle</t>
         </is>
       </c>
       <c r="F190" s="7" t="inlineStr"/>
@@ -5049,12 +5121,12 @@
       </c>
       <c r="D192" s="7" t="inlineStr">
         <is>
+          <t>Ethics</t>
+        </is>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
           <t>Animals</t>
-        </is>
-      </c>
-      <c r="E192" s="7" t="inlineStr">
-        <is>
-          <t>Ethics</t>
         </is>
       </c>
       <c r="F192" s="7" t="inlineStr"/>
@@ -5075,7 +5147,7 @@
       </c>
       <c r="D193" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr"/>
@@ -5141,12 +5213,12 @@
       </c>
       <c r="D196" s="7" t="inlineStr">
         <is>
+          <t>Economy, money, and trade</t>
+        </is>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
           <t>Education</t>
-        </is>
-      </c>
-      <c r="E196" s="7" t="inlineStr">
-        <is>
-          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="F196" s="7" t="inlineStr"/>
@@ -5267,7 +5339,7 @@
       </c>
       <c r="D201" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Government, politics, and diplomacy</t>
         </is>
       </c>
       <c r="E201" s="7" t="inlineStr"/>
@@ -5306,7 +5378,7 @@
       </c>
       <c r="C203" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D203" s="7" t="inlineStr">
@@ -5411,7 +5483,7 @@
       </c>
       <c r="D207" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="E207" s="7" t="inlineStr"/>
@@ -5463,7 +5535,7 @@
       </c>
       <c r="D209" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E209" s="7" t="inlineStr">
@@ -5519,7 +5591,7 @@
       </c>
       <c r="D211" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
@@ -5579,7 +5651,7 @@
       </c>
       <c r="D213" s="7" t="inlineStr">
         <is>
-          <t>Government, politics, and diplomacy</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr"/>
@@ -5596,12 +5668,12 @@
       </c>
       <c r="C214" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D214" s="7" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E214" s="7" t="inlineStr">
@@ -5609,7 +5681,11 @@
           <t>Age, generation, and gender</t>
         </is>
       </c>
-      <c r="F214" s="7" t="inlineStr"/>
+      <c r="F214" s="7" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="5" t="n">
@@ -5617,7 +5693,7 @@
       </c>
       <c r="B215" s="6" t="inlineStr">
         <is>
-          <t>Certain type of music affects young children's learning. Researchers have researched on it. Some people agree and some disagree. What is your opinion?</t>
+          <t>Certain type of music affects young children’s learning. Researchers have researched on it. Some people agree and some disagree. What is your opinion?</t>
         </is>
       </c>
       <c r="C215" s="7" t="inlineStr">
@@ -5627,7 +5703,7 @@
       </c>
       <c r="D215" s="7" t="inlineStr">
         <is>
-          <t>Art and museums</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr"/>
@@ -5639,7 +5715,7 @@
       </c>
       <c r="B216" s="6" t="inlineStr">
         <is>
-          <t>As countries develop, more and more people regard pets as family members. What's your opinion? Support it with examples.</t>
+          <t>As countries develop, more and more people regard pets as family members. What’s your opinion? Support it with examples.</t>
         </is>
       </c>
       <c r="C216" s="7" t="inlineStr">
@@ -5649,11 +5725,19 @@
       </c>
       <c r="D216" s="7" t="inlineStr">
         <is>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E216" s="7" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="F216" s="7" t="inlineStr">
+        <is>
           <t>Animals</t>
         </is>
       </c>
-      <c r="E216" s="7" t="inlineStr"/>
-      <c r="F216" s="7" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="5" t="n">
@@ -5779,7 +5863,7 @@
       </c>
       <c r="D221" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr"/>
@@ -5910,12 +5994,12 @@
       </c>
       <c r="C227" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D227" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Crime, punishment, and law</t>
         </is>
       </c>
       <c r="E227" s="7" t="inlineStr"/>
@@ -5932,12 +6016,12 @@
       </c>
       <c r="C228" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D228" s="7" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Age, generation, and gender</t>
         </is>
       </c>
       <c r="E228" s="7" t="inlineStr"/>
@@ -5985,7 +6069,7 @@
       </c>
       <c r="D230" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E230" s="7" t="inlineStr"/>
@@ -6019,7 +6103,7 @@
       </c>
       <c r="B232" s="6" t="inlineStr">
         <is>
-          <t>Nowadays, with the rapid development of technology, it is easy for people to prepare food. Has it improved the people's quality of life? Discuss it with your own experience.</t>
+          <t>Nowadays, with the rapid development of technology, it is easy for people to prepare food. Has it improved the people’s quality of life? Discuss it with your own experience.</t>
         </is>
       </c>
       <c r="C232" s="7" t="inlineStr">
@@ -6029,7 +6113,7 @@
       </c>
       <c r="D232" s="7" t="inlineStr">
         <is>
-          <t>Food and health</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E232" s="7" t="inlineStr">
@@ -6055,11 +6139,19 @@
       </c>
       <c r="D233" s="7" t="inlineStr">
         <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="E233" s="7" t="inlineStr">
+        <is>
+          <t>Economy, money, and trade</t>
+        </is>
+      </c>
+      <c r="F233" s="7" t="inlineStr">
+        <is>
           <t>City development</t>
         </is>
       </c>
-      <c r="E233" s="7" t="inlineStr"/>
-      <c r="F233" s="7" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="5" t="n">
@@ -6239,7 +6331,7 @@
       </c>
       <c r="D241" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E241" s="7" t="inlineStr"/>
@@ -6261,7 +6353,7 @@
       </c>
       <c r="D242" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E242" s="7" t="inlineStr"/>
@@ -6295,7 +6387,7 @@
       </c>
       <c r="B244" s="6" t="inlineStr">
         <is>
-          <t>People sometimes should do things they aren't willing to do. Discuss whether you agree with this statement or not.</t>
+          <t>People sometimes should do things they aren’t willing to do. Discuss whether you agree with this statement or not.</t>
         </is>
       </c>
       <c r="C244" s="7" t="inlineStr">
@@ -6322,7 +6414,7 @@
       </c>
       <c r="C245" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D245" s="7" t="inlineStr">
@@ -6375,15 +6467,19 @@
       </c>
       <c r="D247" s="7" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
-        </is>
-      </c>
-      <c r="F247" s="7" t="inlineStr"/>
+          <t>Age, generation, and gender</t>
+        </is>
+      </c>
+      <c r="F247" s="7" t="inlineStr">
+        <is>
+          <t>Travelling and tourism</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="5" t="n">
@@ -6401,7 +6497,7 @@
       </c>
       <c r="D248" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="E248" s="7" t="inlineStr"/>
@@ -6445,7 +6541,7 @@
       </c>
       <c r="D250" s="7" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
+          <t>Art and museums</t>
         </is>
       </c>
       <c r="E250" s="7" t="inlineStr"/>
@@ -6467,11 +6563,19 @@
       </c>
       <c r="D251" s="7" t="inlineStr">
         <is>
-          <t>Food and health</t>
-        </is>
-      </c>
-      <c r="E251" s="7" t="inlineStr"/>
-      <c r="F251" s="7" t="inlineStr"/>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E251" s="7" t="inlineStr">
+        <is>
+          <t>Science, technology, and innovation</t>
+        </is>
+      </c>
+      <c r="F251" s="7" t="inlineStr">
+        <is>
+          <t>Ethics</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="5" t="n">
@@ -6511,7 +6615,7 @@
       </c>
       <c r="D253" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E253" s="7" t="inlineStr"/>
@@ -6533,12 +6637,12 @@
       </c>
       <c r="D254" s="7" t="inlineStr">
         <is>
-          <t>Animals</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E254" s="7" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>City development</t>
         </is>
       </c>
       <c r="F254" s="7" t="inlineStr">
@@ -6585,12 +6689,12 @@
       </c>
       <c r="D256" s="7" t="inlineStr">
         <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="E256" s="7" t="inlineStr">
+        <is>
           <t>Age, generation, and gender</t>
-        </is>
-      </c>
-      <c r="E256" s="7" t="inlineStr">
-        <is>
-          <t>Lifestyle</t>
         </is>
       </c>
       <c r="F256" s="7" t="inlineStr"/>
@@ -6611,7 +6715,7 @@
       </c>
       <c r="D257" s="7" t="inlineStr">
         <is>
-          <t>Economy, money, and trade</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E257" s="7" t="inlineStr"/>
@@ -6654,7 +6758,7 @@
       </c>
       <c r="C259" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D259" s="7" t="inlineStr">
@@ -6703,7 +6807,7 @@
       </c>
       <c r="D261" s="7" t="inlineStr">
         <is>
-          <t>Art and museums</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E261" s="7" t="inlineStr"/>
@@ -6769,7 +6873,7 @@
       </c>
       <c r="D264" s="7" t="inlineStr">
         <is>
-          <t>Travelling and tourism</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E264" s="7" t="inlineStr"/>
@@ -6791,11 +6895,19 @@
       </c>
       <c r="D265" s="7" t="inlineStr">
         <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="E265" s="7" t="inlineStr"/>
-      <c r="F265" s="7" t="inlineStr"/>
+          <t>Crime, punishment, and law</t>
+        </is>
+      </c>
+      <c r="E265" s="7" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="F265" s="7" t="inlineStr">
+        <is>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="5" t="n">
@@ -6861,7 +6973,7 @@
       </c>
       <c r="D268" s="7" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Age, generation, and gender</t>
         </is>
       </c>
       <c r="E268" s="7" t="inlineStr"/>
@@ -6905,7 +7017,7 @@
       </c>
       <c r="D270" s="7" t="inlineStr">
         <is>
-          <t>Government, politics, and diplomacy</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="E270" s="7" t="inlineStr"/>
@@ -6927,7 +7039,7 @@
       </c>
       <c r="D271" s="7" t="inlineStr">
         <is>
-          <t>Crime, punishment, and law</t>
+          <t>Ethics</t>
         </is>
       </c>
       <c r="E271" s="7" t="inlineStr"/>
@@ -6949,7 +7061,7 @@
       </c>
       <c r="D272" s="7" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E272" s="7" t="inlineStr"/>
@@ -6983,12 +7095,12 @@
       </c>
       <c r="B274" s="6" t="inlineStr">
         <is>
-          <t>Some people think that the automobile has improved modern life. Others think that the automobile has caused serious problems. What's your opinion about it?</t>
+          <t>Some people think that the automobile has improved modern life. Others think that the automobile has caused serious problems. What’s your opinion about it?</t>
         </is>
       </c>
       <c r="C274" s="7" t="inlineStr">
         <is>
-          <t>To what extent do you agree or disagree</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D274" s="7" t="inlineStr">
@@ -7062,8 +7174,16 @@
           <t>Food and health</t>
         </is>
       </c>
-      <c r="E277" s="7" t="inlineStr"/>
-      <c r="F277" s="7" t="inlineStr"/>
+      <c r="E277" s="7" t="inlineStr">
+        <is>
+          <t>Ethics</t>
+        </is>
+      </c>
+      <c r="F277" s="7" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="5" t="n">
@@ -7103,7 +7223,7 @@
       </c>
       <c r="D279" s="7" t="inlineStr">
         <is>
-          <t>Travelling and tourism</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E279" s="7" t="inlineStr"/>
@@ -7125,7 +7245,7 @@
       </c>
       <c r="D280" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="E280" s="7" t="inlineStr"/>
@@ -7142,12 +7262,12 @@
       </c>
       <c r="C281" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D281" s="7" t="inlineStr">
         <is>
-          <t>Economy, money, and trade</t>
+          <t>Leisure, sports, and hobbies</t>
         </is>
       </c>
       <c r="E281" s="7" t="inlineStr"/>
@@ -7186,12 +7306,12 @@
       </c>
       <c r="C283" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D283" s="7" t="inlineStr">
         <is>
-          <t>Socio-cultural and global issues</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="E283" s="7" t="inlineStr"/>
@@ -7208,12 +7328,12 @@
       </c>
       <c r="C284" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D284" s="7" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
+          <t>Crime, punishment, and law</t>
         </is>
       </c>
       <c r="E284" s="7" t="inlineStr"/>
@@ -7230,12 +7350,12 @@
       </c>
       <c r="C285" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D285" s="7" t="inlineStr">
         <is>
-          <t>Food and health</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E285" s="7" t="inlineStr"/>
@@ -7257,7 +7377,7 @@
       </c>
       <c r="D286" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E286" s="7" t="inlineStr">
@@ -7265,7 +7385,11 @@
           <t>Population</t>
         </is>
       </c>
-      <c r="F286" s="7" t="inlineStr"/>
+      <c r="F286" s="7" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="5" t="n">
@@ -7278,7 +7402,7 @@
       </c>
       <c r="C287" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D287" s="7" t="inlineStr">
@@ -7331,7 +7455,7 @@
       </c>
       <c r="D289" s="7" t="inlineStr">
         <is>
-          <t>Food and health</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="E289" s="7" t="inlineStr"/>
@@ -7397,7 +7521,7 @@
       </c>
       <c r="D292" s="7" t="inlineStr">
         <is>
-          <t>Animals</t>
+          <t>Ethics</t>
         </is>
       </c>
       <c r="E292" s="7" t="inlineStr">
@@ -7427,7 +7551,7 @@
       </c>
       <c r="D293" s="7" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E293" s="7" t="inlineStr"/>
@@ -7523,7 +7647,7 @@
       </c>
       <c r="D297" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E297" s="7" t="inlineStr"/>
@@ -7567,7 +7691,7 @@
       </c>
       <c r="D299" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Leisure, sports, and hobbies</t>
         </is>
       </c>
       <c r="E299" s="7" t="inlineStr"/>
@@ -7579,7 +7703,7 @@
       </c>
       <c r="B300" s="6" t="inlineStr">
         <is>
-          <t>A gift (such as a camera, a soccer ball, or an animal) can contribute to a child's development. What gift would you give to help a child develop? Why do you choose it?</t>
+          <t>A gift (such as a camera, a soccer ball, or an animal) can contribute to a child’s development. What gift would you give to help a child develop? Why do you choose it?</t>
         </is>
       </c>
       <c r="C300" s="7" t="inlineStr">
@@ -7589,7 +7713,7 @@
       </c>
       <c r="D300" s="7" t="inlineStr">
         <is>
-          <t>Animals</t>
+          <t>Leisure, sports, and hobbies</t>
         </is>
       </c>
       <c r="E300" s="7" t="inlineStr"/>
@@ -7606,12 +7730,12 @@
       </c>
       <c r="C301" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D301" s="7" t="inlineStr">
         <is>
-          <t>Travelling and tourism</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E301" s="7" t="inlineStr"/>
@@ -7689,7 +7813,7 @@
       </c>
       <c r="B305" s="6" t="inlineStr">
         <is>
-          <t>How do movies or television influence people's behavior?</t>
+          <t>How do movies or television influence people’s behavior?</t>
         </is>
       </c>
       <c r="C305" s="7" t="inlineStr">
@@ -7699,7 +7823,7 @@
       </c>
       <c r="D305" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E305" s="7" t="inlineStr"/>
@@ -7721,15 +7845,19 @@
       </c>
       <c r="D306" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E306" s="7" t="inlineStr">
         <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="F306" s="7" t="inlineStr">
+        <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="F306" s="7" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" s="5" t="n">
@@ -7747,7 +7875,7 @@
       </c>
       <c r="D307" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E307" s="7" t="inlineStr"/>
@@ -7781,7 +7909,7 @@
       </c>
       <c r="B309" s="6" t="inlineStr">
         <is>
-          <t>Choose one transportation vehicle and explain why you think it has changed people's lives.</t>
+          <t>Choose one transportation vehicle and explain why you think it has changed people’s lives.</t>
         </is>
       </c>
       <c r="C309" s="7" t="inlineStr">
@@ -7791,7 +7919,7 @@
       </c>
       <c r="D309" s="7" t="inlineStr">
         <is>
-          <t>Traffic</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E309" s="7" t="inlineStr"/>
@@ -7835,10 +7963,14 @@
       </c>
       <c r="D311" s="7" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
-        </is>
-      </c>
-      <c r="E311" s="7" t="inlineStr"/>
+          <t>Ethics</t>
+        </is>
+      </c>
+      <c r="E311" s="7" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
       <c r="F311" s="7" t="inlineStr"/>
     </row>
     <row r="312">
@@ -7857,17 +7989,17 @@
       </c>
       <c r="D312" s="7" t="inlineStr">
         <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="E312" s="7" t="inlineStr">
+        <is>
+          <t>Economy, money, and trade</t>
+        </is>
+      </c>
+      <c r="F312" s="7" t="inlineStr">
+        <is>
           <t>Animals</t>
-        </is>
-      </c>
-      <c r="E312" s="7" t="inlineStr">
-        <is>
-          <t>Environment</t>
-        </is>
-      </c>
-      <c r="F312" s="7" t="inlineStr">
-        <is>
-          <t>Ethics</t>
         </is>
       </c>
     </row>
@@ -7909,7 +8041,7 @@
       </c>
       <c r="D314" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E314" s="7" t="inlineStr"/>
@@ -7921,7 +8053,7 @@
       </c>
       <c r="B315" s="6" t="inlineStr">
         <is>
-          <t>Some people prefer to get up early in the morning and start the day's work. Others prefer to get up later in the day and work until late at night. Which do you prefer? Explain it with your own experience.</t>
+          <t>Some people prefer to get up early in the morning and start the day’s work. Others prefer to get up later in the day and work until late at night. Which do you prefer? Explain it with your own experience.</t>
         </is>
       </c>
       <c r="C315" s="7" t="inlineStr">
@@ -7931,7 +8063,7 @@
       </c>
       <c r="D315" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E315" s="7" t="inlineStr"/>
@@ -7970,7 +8102,7 @@
       </c>
       <c r="C317" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D317" s="7" t="inlineStr">
@@ -8113,7 +8245,7 @@
       </c>
       <c r="D322" s="7" t="inlineStr">
         <is>
-          <t>Crime, punishment, and law</t>
+          <t>Ethics</t>
         </is>
       </c>
       <c r="E322" s="7" t="inlineStr"/>
@@ -8243,7 +8375,7 @@
       </c>
       <c r="B328" s="6" t="inlineStr">
         <is>
-          <t>Classmates have a more important influence than parents on a child's success in school. To what extent do you agree with this statement?</t>
+          <t>Classmates have a more important influence than parents on a child’s success in school. To what extent do you agree with this statement?</t>
         </is>
       </c>
       <c r="C328" s="7" t="inlineStr">
@@ -8279,7 +8411,7 @@
       </c>
       <c r="D329" s="7" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E329" s="7" t="inlineStr"/>
@@ -8323,7 +8455,7 @@
       </c>
       <c r="D331" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E331" s="7" t="inlineStr"/>
@@ -8367,12 +8499,12 @@
       </c>
       <c r="D333" s="7" t="inlineStr">
         <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E333" s="7" t="inlineStr">
+        <is>
           <t>Language</t>
-        </is>
-      </c>
-      <c r="E333" s="7" t="inlineStr">
-        <is>
-          <t>Education</t>
         </is>
       </c>
       <c r="F333" s="7" t="inlineStr">
@@ -8397,7 +8529,7 @@
       </c>
       <c r="D334" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E334" s="7" t="inlineStr"/>
@@ -8463,12 +8595,12 @@
       </c>
       <c r="D337" s="7" t="inlineStr">
         <is>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E337" s="7" t="inlineStr">
+        <is>
           <t>Age, generation, and gender</t>
-        </is>
-      </c>
-      <c r="E337" s="7" t="inlineStr">
-        <is>
-          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="F337" s="7" t="inlineStr">
@@ -8537,7 +8669,7 @@
       </c>
       <c r="D340" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E340" s="7" t="inlineStr"/>
@@ -8611,7 +8743,7 @@
       </c>
       <c r="D343" s="7" t="inlineStr">
         <is>
-          <t>Food and health</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E343" s="7" t="inlineStr">
@@ -8654,12 +8786,12 @@
       </c>
       <c r="C345" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D345" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E345" s="7" t="inlineStr"/>
@@ -8671,7 +8803,7 @@
       </c>
       <c r="B346" s="6" t="inlineStr">
         <is>
-          <t>Movies and television have a bad influence on people's behaviors. To what extent do you agree with this statement?</t>
+          <t>Movies and television have a bad influence on people’s behaviors. To what extent do you agree with this statement?</t>
         </is>
       </c>
       <c r="C346" s="7" t="inlineStr">
@@ -8681,7 +8813,7 @@
       </c>
       <c r="D346" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E346" s="7" t="inlineStr"/>
@@ -8725,7 +8857,7 @@
       </c>
       <c r="D348" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E348" s="7" t="inlineStr"/>
@@ -8747,7 +8879,7 @@
       </c>
       <c r="D349" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E349" s="7" t="inlineStr"/>
@@ -8759,7 +8891,7 @@
       </c>
       <c r="B350" s="6" t="inlineStr">
         <is>
-          <t>Universities should give the same amount of money to their students' sports activities as they give to their university libraries. Do you agree or disagree with the statement?</t>
+          <t>Universities should give the same amount of money to their students’ sports activities as they give to their university libraries. Do you agree or disagree with the statement?</t>
         </is>
       </c>
       <c r="C350" s="7" t="inlineStr">
@@ -8861,10 +8993,14 @@
       </c>
       <c r="D354" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
-        </is>
-      </c>
-      <c r="E354" s="7" t="inlineStr"/>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E354" s="7" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
       <c r="F354" s="7" t="inlineStr"/>
     </row>
     <row r="355">
@@ -8883,7 +9019,7 @@
       </c>
       <c r="D355" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E355" s="7" t="inlineStr">
@@ -8904,7 +9040,7 @@
       </c>
       <c r="C356" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D356" s="7" t="inlineStr">
@@ -8912,8 +9048,16 @@
           <t>Population</t>
         </is>
       </c>
-      <c r="E356" s="7" t="inlineStr"/>
-      <c r="F356" s="7" t="inlineStr"/>
+      <c r="E356" s="7" t="inlineStr">
+        <is>
+          <t>Food and health</t>
+        </is>
+      </c>
+      <c r="F356" s="7" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="5" t="n">
@@ -8931,7 +9075,7 @@
       </c>
       <c r="D357" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E357" s="7" t="inlineStr"/>
@@ -8979,7 +9123,7 @@
       </c>
       <c r="D359" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E359" s="7" t="inlineStr"/>
@@ -9001,7 +9145,7 @@
       </c>
       <c r="D360" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="E360" s="7" t="inlineStr"/>
@@ -9018,7 +9162,7 @@
       </c>
       <c r="C361" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D361" s="7" t="inlineStr">
@@ -9071,7 +9215,7 @@
       </c>
       <c r="D363" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E363" s="7" t="inlineStr"/>
@@ -9093,11 +9237,19 @@
       </c>
       <c r="D364" s="7" t="inlineStr">
         <is>
+          <t>Ethics</t>
+        </is>
+      </c>
+      <c r="E364" s="7" t="inlineStr">
+        <is>
           <t>Economy, money, and trade</t>
         </is>
       </c>
-      <c r="E364" s="7" t="inlineStr"/>
-      <c r="F364" s="7" t="inlineStr"/>
+      <c r="F364" s="7" t="inlineStr">
+        <is>
+          <t>Work</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="5" t="n">
@@ -9189,7 +9341,7 @@
       </c>
       <c r="D368" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="E368" s="7" t="inlineStr"/>
@@ -9211,7 +9363,7 @@
       </c>
       <c r="D369" s="7" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E369" s="7" t="inlineStr"/>
@@ -9223,7 +9375,7 @@
       </c>
       <c r="B370" s="6" t="inlineStr">
         <is>
-          <t>Scientists have been debating the impact of nature and nurture on people's personality and behavior. Nature brings you inborn skills and nurture helps you obtain skills by practices. Which one do you think has a greater influence?</t>
+          <t>Scientists have been debating the impact of nature and nurture on people’s personality and behavior. Nature brings you inborn skills and nurture helps you obtain skills by practices. Which one do you think has a greater influence?</t>
         </is>
       </c>
       <c r="C370" s="7" t="inlineStr">
@@ -9233,7 +9385,7 @@
       </c>
       <c r="D370" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E370" s="7" t="inlineStr"/>
@@ -9281,7 +9433,7 @@
       </c>
       <c r="D372" s="7" t="inlineStr">
         <is>
-          <t>Traffic</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E372" s="7" t="inlineStr"/>
@@ -9303,7 +9455,7 @@
       </c>
       <c r="D373" s="7" t="inlineStr">
         <is>
-          <t>Art and museums</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E373" s="7" t="inlineStr">
@@ -9355,7 +9507,7 @@
       </c>
       <c r="D375" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E375" s="7" t="inlineStr"/>
@@ -9372,7 +9524,7 @@
       </c>
       <c r="C376" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D376" s="7" t="inlineStr">
@@ -9380,8 +9532,16 @@
           <t>Media and communication</t>
         </is>
       </c>
-      <c r="E376" s="7" t="inlineStr"/>
-      <c r="F376" s="7" t="inlineStr"/>
+      <c r="E376" s="7" t="inlineStr">
+        <is>
+          <t>Food and health</t>
+        </is>
+      </c>
+      <c r="F376" s="7" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="5" t="n">
@@ -9399,7 +9559,7 @@
       </c>
       <c r="D377" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E377" s="7" t="inlineStr"/>
@@ -9421,11 +9581,19 @@
       </c>
       <c r="D378" s="7" t="inlineStr">
         <is>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E378" s="7" t="inlineStr">
+        <is>
+          <t>Food and health</t>
+        </is>
+      </c>
+      <c r="F378" s="7" t="inlineStr">
+        <is>
           <t>Media and communication</t>
         </is>
       </c>
-      <c r="E378" s="7" t="inlineStr"/>
-      <c r="F378" s="7" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" s="5" t="n">
@@ -9487,7 +9655,7 @@
       </c>
       <c r="D381" s="7" t="inlineStr">
         <is>
-          <t>Science, technology, and innovation</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E381" s="7" t="inlineStr"/>
@@ -9552,7 +9720,7 @@
       </c>
       <c r="C384" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D384" s="7" t="inlineStr">
@@ -9579,7 +9747,7 @@
       </c>
       <c r="D385" s="7" t="inlineStr">
         <is>
-          <t>Media and communication</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E385" s="7" t="inlineStr"/>
@@ -9601,7 +9769,7 @@
       </c>
       <c r="D386" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E386" s="7" t="inlineStr"/>
@@ -9623,11 +9791,19 @@
       </c>
       <c r="D387" s="7" t="inlineStr">
         <is>
-          <t>Science, technology, and innovation</t>
-        </is>
-      </c>
-      <c r="E387" s="7" t="inlineStr"/>
-      <c r="F387" s="7" t="inlineStr"/>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E387" s="7" t="inlineStr">
+        <is>
+          <t>Media and communication</t>
+        </is>
+      </c>
+      <c r="F387" s="7" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="5" t="n">
@@ -9662,7 +9838,7 @@
       </c>
       <c r="C389" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D389" s="7" t="inlineStr">
@@ -9759,7 +9935,7 @@
       </c>
       <c r="D393" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Ethics</t>
         </is>
       </c>
       <c r="E393" s="7" t="inlineStr"/>
@@ -9851,7 +10027,7 @@
       </c>
       <c r="D397" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E397" s="7" t="inlineStr"/>
@@ -9873,7 +10049,7 @@
       </c>
       <c r="D398" s="7" t="inlineStr">
         <is>
-          <t>Science, technology, and innovation</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E398" s="7" t="inlineStr"/>
@@ -9917,7 +10093,7 @@
       </c>
       <c r="D400" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E400" s="7" t="inlineStr"/>
@@ -9934,7 +10110,7 @@
       </c>
       <c r="C401" s="7" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D401" s="7" t="inlineStr">
@@ -9969,11 +10145,19 @@
       </c>
       <c r="D402" s="7" t="inlineStr">
         <is>
+          <t>Media and communication</t>
+        </is>
+      </c>
+      <c r="E402" s="7" t="inlineStr">
+        <is>
           <t>Science, technology, and innovation</t>
         </is>
       </c>
-      <c r="E402" s="7" t="inlineStr"/>
-      <c r="F402" s="7" t="inlineStr"/>
+      <c r="F402" s="7" t="inlineStr">
+        <is>
+          <t>Leisure, sports, and hobbies</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="5" t="n">
@@ -9991,15 +10175,19 @@
       </c>
       <c r="D403" s="7" t="inlineStr">
         <is>
+          <t>Food and health</t>
+        </is>
+      </c>
+      <c r="E403" s="7" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="F403" s="7" t="inlineStr">
+        <is>
           <t>Climate</t>
         </is>
       </c>
-      <c r="E403" s="7" t="inlineStr">
-        <is>
-          <t>Environment</t>
-        </is>
-      </c>
-      <c r="F403" s="7" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" s="5" t="n">
@@ -10017,7 +10205,7 @@
       </c>
       <c r="D404" s="7" t="inlineStr">
         <is>
-          <t>Government, politics, and diplomacy</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E404" s="7" t="inlineStr"/>
@@ -10039,7 +10227,7 @@
       </c>
       <c r="D405" s="7" t="inlineStr">
         <is>
-          <t>Traffic</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E405" s="7" t="inlineStr"/>
@@ -10061,7 +10249,7 @@
       </c>
       <c r="D406" s="7" t="inlineStr">
         <is>
-          <t>Science, technology, and innovation</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="E406" s="7" t="inlineStr"/>
@@ -10113,11 +10301,19 @@
       </c>
       <c r="D408" s="7" t="inlineStr">
         <is>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
+      <c r="E408" s="7" t="inlineStr">
+        <is>
           <t>Media and communication</t>
         </is>
       </c>
-      <c r="E408" s="7" t="inlineStr"/>
-      <c r="F408" s="7" t="inlineStr"/>
+      <c r="F408" s="7" t="inlineStr">
+        <is>
+          <t>Ethics</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" s="5" t="n">
@@ -10135,7 +10331,7 @@
       </c>
       <c r="D409" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E409" s="7" t="inlineStr"/>
@@ -10179,10 +10375,14 @@
       </c>
       <c r="D411" s="7" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
-        </is>
-      </c>
-      <c r="E411" s="7" t="inlineStr"/>
+          <t>Science, technology, and innovation</t>
+        </is>
+      </c>
+      <c r="E411" s="7" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
       <c r="F411" s="7" t="inlineStr"/>
     </row>
     <row r="412">
@@ -10201,7 +10401,7 @@
       </c>
       <c r="D412" s="7" t="inlineStr">
         <is>
-          <t>Animals</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="E412" s="7" t="inlineStr"/>
@@ -10223,7 +10423,7 @@
       </c>
       <c r="D413" s="7" t="inlineStr">
         <is>
-          <t>Science, technology, and innovation</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="E413" s="7" t="inlineStr"/>
@@ -10245,7 +10445,7 @@
       </c>
       <c r="D414" s="7" t="inlineStr">
         <is>
-          <t>Traffic</t>
+          <t>City development</t>
         </is>
       </c>
       <c r="E414" s="7" t="inlineStr"/>
@@ -10311,7 +10511,7 @@
       </c>
       <c r="D417" s="7" t="inlineStr">
         <is>
-          <t>Travelling and tourism</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="E417" s="7" t="inlineStr"/>
@@ -10333,7 +10533,7 @@
       </c>
       <c r="D418" s="7" t="inlineStr">
         <is>
-          <t>Traffic</t>
+          <t>City development</t>
         </is>
       </c>
       <c r="E418" s="7" t="inlineStr">
@@ -10385,7 +10585,7 @@
       </c>
       <c r="D420" s="7" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E420" s="7" t="inlineStr">
@@ -10393,7 +10593,11 @@
           <t>Food and health</t>
         </is>
       </c>
-      <c r="F420" s="7" t="inlineStr"/>
+      <c r="F420" s="7" t="inlineStr">
+        <is>
+          <t>Science, technology, and innovation</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" s="5" t="n">
@@ -10411,7 +10615,7 @@
       </c>
       <c r="D421" s="7" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Ethics</t>
         </is>
       </c>
       <c r="E421" s="7" t="inlineStr">
@@ -10437,7 +10641,7 @@
       </c>
       <c r="D422" s="7" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E422" s="7" t="inlineStr"/>
@@ -10459,7 +10663,7 @@
       </c>
       <c r="D423" s="7" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Food and health</t>
         </is>
       </c>
       <c r="E423" s="7" t="inlineStr"/>
@@ -10481,7 +10685,7 @@
       </c>
       <c r="D424" s="7" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Lifestyle</t>
         </is>
       </c>
       <c r="E424" s="7" t="inlineStr"/>
@@ -10503,7 +10707,7 @@
       </c>
       <c r="D425" s="7" t="inlineStr">
         <is>
-          <t>Media and communication</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E425" s="7" t="inlineStr"/>
@@ -10525,7 +10729,7 @@
       </c>
       <c r="D426" s="7" t="inlineStr">
         <is>
-          <t>Animals</t>
+          <t>Ethics</t>
         </is>
       </c>
       <c r="E426" s="7" t="inlineStr"/>
@@ -10547,7 +10751,7 @@
       </c>
       <c r="D427" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Food and health</t>
         </is>
       </c>
       <c r="E427" s="7" t="inlineStr"/>
@@ -10598,8 +10802,16 @@
           <t>Government, politics, and diplomacy</t>
         </is>
       </c>
-      <c r="E429" s="7" t="inlineStr"/>
-      <c r="F429" s="7" t="inlineStr"/>
+      <c r="E429" s="7" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="F429" s="7" t="inlineStr">
+        <is>
+          <t>Science, technology, and innovation</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" s="5" t="n">
@@ -10617,7 +10829,7 @@
       </c>
       <c r="D430" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Ethics</t>
         </is>
       </c>
       <c r="E430" s="7" t="inlineStr"/>
@@ -10639,7 +10851,7 @@
       </c>
       <c r="D431" s="7" t="inlineStr">
         <is>
-          <t>Media and communication</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="E431" s="7" t="inlineStr"/>
@@ -10835,7 +11047,7 @@
       </c>
       <c r="D439" s="7" t="inlineStr">
         <is>
-          <t>Art and museums</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E439" s="7" t="inlineStr"/>
@@ -10860,8 +11072,16 @@
           <t>Government, politics, and diplomacy</t>
         </is>
       </c>
-      <c r="E440" s="7" t="inlineStr"/>
-      <c r="F440" s="7" t="inlineStr"/>
+      <c r="E440" s="7" t="inlineStr">
+        <is>
+          <t>Science, technology, and innovation</t>
+        </is>
+      </c>
+      <c r="F440" s="7" t="inlineStr">
+        <is>
+          <t>Ethics</t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" s="5" t="n">
@@ -10879,7 +11099,7 @@
       </c>
       <c r="D441" s="7" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Food and health</t>
         </is>
       </c>
       <c r="E441" s="7" t="inlineStr"/>
@@ -10923,7 +11143,7 @@
       </c>
       <c r="D443" s="7" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E443" s="7" t="inlineStr"/>
@@ -10967,7 +11187,7 @@
       </c>
       <c r="D445" s="7" t="inlineStr">
         <is>
-          <t>Lifestyle</t>
+          <t>Food and health</t>
         </is>
       </c>
       <c r="E445" s="7" t="inlineStr"/>
@@ -11015,7 +11235,7 @@
       </c>
       <c r="D447" s="7" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>Food and health</t>
         </is>
       </c>
       <c r="E447" s="7" t="inlineStr"/>
@@ -11040,8 +11260,16 @@
           <t>Media and communication</t>
         </is>
       </c>
-      <c r="E448" s="7" t="inlineStr"/>
-      <c r="F448" s="7" t="inlineStr"/>
+      <c r="E448" s="7" t="inlineStr">
+        <is>
+          <t>Ethics</t>
+        </is>
+      </c>
+      <c r="F448" s="7" t="inlineStr">
+        <is>
+          <t>Socio-cultural and global issues</t>
+        </is>
+      </c>
     </row>
     <row r="449">
       <c r="A449" s="5" t="n">
@@ -11081,7 +11309,7 @@
       </c>
       <c r="D450" s="7" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="E450" s="7" t="inlineStr"/>
@@ -11147,7 +11375,7 @@
       </c>
       <c r="D453" s="7" t="inlineStr">
         <is>
-          <t>Animals</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E453" s="7" t="inlineStr"/>
@@ -11169,12 +11397,12 @@
       </c>
       <c r="D454" s="7" t="inlineStr">
         <is>
+          <t>Science, technology, and innovation</t>
+        </is>
+      </c>
+      <c r="E454" s="7" t="inlineStr">
+        <is>
           <t>Ethics</t>
-        </is>
-      </c>
-      <c r="E454" s="7" t="inlineStr">
-        <is>
-          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="F454" s="7" t="inlineStr"/>
@@ -11195,7 +11423,7 @@
       </c>
       <c r="D455" s="7" t="inlineStr">
         <is>
-          <t>Science, technology, and innovation</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E455" s="7" t="inlineStr"/>
@@ -11217,7 +11445,7 @@
       </c>
       <c r="D456" s="7" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="E456" s="7" t="inlineStr">
@@ -11242,12 +11470,12 @@
       </c>
       <c r="C457" s="7" t="inlineStr">
         <is>
-          <t>Do the advantages outweigh the disadvantages</t>
+          <t>others</t>
         </is>
       </c>
       <c r="D457" s="7" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="E457" s="7" t="inlineStr"/>
@@ -11412,7 +11640,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Media and communication</t>
+          <t>Socio-cultural and global issues</t>
         </is>
       </c>
       <c r="C6" s="14">
@@ -11452,7 +11680,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>Science, technology, and innovation</t>
         </is>
       </c>
       <c r="C7" s="14">
@@ -11495,7 +11723,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Age, generation, and gender</t>
+          <t>Media and communication</t>
         </is>
       </c>
       <c r="C8" s="14">
@@ -11581,7 +11809,7 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>City development</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="C10" s="14">
@@ -11624,7 +11852,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Leisure, sports, and hobbies</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="C11" s="14">
@@ -11667,7 +11895,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Science, technology, and innovation</t>
+          <t>Economy, money, and trade</t>
         </is>
       </c>
       <c r="C12" s="14">
@@ -11701,7 +11929,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Age, generation, and gender</t>
         </is>
       </c>
       <c r="C13" s="14">
@@ -11735,7 +11963,7 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Socio-cultural and global issues</t>
+          <t>Food and health</t>
         </is>
       </c>
       <c r="C14" s="14">
@@ -11769,7 +11997,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Economy, money, and trade</t>
+          <t>Leisure, sports, and hobbies</t>
         </is>
       </c>
       <c r="C15" s="14">
@@ -11803,7 +12031,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Ethics</t>
+          <t>City development</t>
         </is>
       </c>
       <c r="C16" s="14">
@@ -11837,7 +12065,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Food and health</t>
+          <t>Ethics</t>
         </is>
       </c>
       <c r="C17" s="14">
@@ -11871,7 +12099,7 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Government, politics, and diplomacy</t>
         </is>
       </c>
       <c r="C18" s="14">
@@ -11905,7 +12133,7 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Travelling and tourism</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="C19" s="14">
@@ -11939,7 +12167,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Crime, punishment, and law</t>
         </is>
       </c>
       <c r="C20" s="14">
@@ -11973,7 +12201,7 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Traffic</t>
+          <t>Travelling and tourism</t>
         </is>
       </c>
       <c r="C21" s="14">
@@ -12007,7 +12235,7 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Animals</t>
+          <t>Climate</t>
         </is>
       </c>
       <c r="C22" s="14">
@@ -12041,7 +12269,7 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Government, politics, and diplomacy</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="C23" s="14">
@@ -12109,7 +12337,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Animals</t>
         </is>
       </c>
       <c r="C25" s="14">
@@ -12143,7 +12371,7 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Crime, punishment, and law</t>
+          <t>Traffic</t>
         </is>
       </c>
       <c r="C26" s="14">
@@ -12325,7 +12553,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>causes-problems-solutions</t>
+          <t>Is it a positive or negative development</t>
         </is>
       </c>
       <c r="C8" s="14">
@@ -12343,7 +12571,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Is it a positive or negative development</t>
+          <t>causes-problems-solutions</t>
         </is>
       </c>
       <c r="C9" s="14">

</xml_diff>

<commit_message>
release: V1.8.84 - Vocab Book UI Rework, Track Progress Redesign, and V4 Review UI Modernization
</commit_message>
<xml_diff>
--- a/public/database/Write Essay/PTE_453_Cleaned_Prompts_Topics_Task_Types.xlsx
+++ b/public/database/Write Essay/PTE_453_Cleaned_Prompts_Topics_Task_Types.xlsx
@@ -81,7 +81,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -125,11 +125,44 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,6 +210,7 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -543,7 +577,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F457"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="82" customWidth="1" min="2" max="2"/>
@@ -9425,10 +9459,14 @@
       <c r="A372" s="5" t="n">
         <v>370</v>
       </c>
-      <c r="B372" s="6" t="inlineStr"/>
+      <c r="B372" s="6" t="inlineStr">
+        <is>
+          <t>It is important to look at the positive aspects when discussing various subjects. Do you agree or disagree? Give reasons and examples to support your view.</t>
+        </is>
+      </c>
       <c r="C372" s="7" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>To what extent do you agree or disagree</t>
         </is>
       </c>
       <c r="D372" s="7" t="inlineStr">
@@ -11497,7 +11535,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -11523,7 +11561,7 @@
           <t>Model inputs</t>
         </is>
       </c>
-      <c r="K1" s="9" t="n"/>
+      <c r="K1" s="23" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -11672,7 +11710,7 @@
           <t>Key results</t>
         </is>
       </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="K6" s="23" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="13" t="n">
@@ -12449,7 +12487,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
feat(write-essay): publish 453 multi-model audited guided support packs (task 726)
</commit_message>
<xml_diff>
--- a/public/database/Write Essay/PTE_453_Cleaned_Prompts_Topics_Task_Types.xlsx
+++ b/public/database/Write Essay/PTE_453_Cleaned_Prompts_Topics_Task_Types.xlsx
@@ -81,7 +81,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -125,11 +125,44 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,6 +210,7 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -543,7 +577,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F457"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="82" customWidth="1" min="2" max="2"/>
@@ -9425,10 +9459,14 @@
       <c r="A372" s="5" t="n">
         <v>370</v>
       </c>
-      <c r="B372" s="6" t="inlineStr"/>
+      <c r="B372" s="6" t="inlineStr">
+        <is>
+          <t>It is important to look at the positive aspects when discussing various subjects. Do you agree or disagree? Give reasons and examples to support your view.</t>
+        </is>
+      </c>
       <c r="C372" s="7" t="inlineStr">
         <is>
-          <t>others</t>
+          <t>To what extent do you agree or disagree</t>
         </is>
       </c>
       <c r="D372" s="7" t="inlineStr">
@@ -11497,7 +11535,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -11523,7 +11561,7 @@
           <t>Model inputs</t>
         </is>
       </c>
-      <c r="K1" s="9" t="n"/>
+      <c r="K1" s="23" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -11672,7 +11710,7 @@
           <t>Key results</t>
         </is>
       </c>
-      <c r="K6" s="9" t="n"/>
+      <c r="K6" s="23" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="13" t="n">
@@ -12449,7 +12487,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>

</xml_diff>